<commit_message>
Record the chart pop-up change in the development plan
The specification carried it at v1.16; the plan did not, and the plan is where the
version history lives - it already records UI changes at this grain, including the
shell chrome overlap in v2.41. v2.42 adds R-34: what was missing from the project
chart's pop-up, why the total is summed over every project in view rather than over
the bands drawn, and the two checks test_charts.py gained.

No register row for R-34. That register was frozen at the Gate 1 baseline and stops at
R-13; R-14 onward - R-30, R-31, R-32, R-33 among them - are carried in the version
history and cited from the requirement rows, which is the established pattern.

Plan v2.42, specification v1.16 (now citing it), app v1.40, guide and contract rebuilt
against it. All 28 suites pass; check_consistency reports no problems.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XSm1KSGtymAaRV3ZhUyDkk
</commit_message>
<xml_diff>
--- a/docs/PRAP_Programming_Specification_v1.16.xlsx
+++ b/docs/PRAP_Programming_Specification_v1.16.xlsx
@@ -627,7 +627,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>PRAP_Development_Plan_v2.41.xlsx - APPROVED BASELINE, Dan 2026-08-02</t>
+          <t>PRAP_Development_Plan_v2.42.xlsx - APPROVED BASELINE, Dan 2026-08-02</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Read directly from PRAP_Development_Plan_v2.41.xlsx sheet 03, so a requirement cannot be lost between the two documents.</t>
+          <t>Read directly from PRAP_Development_Plan_v2.42.xlsx sheet 03, so a requirement cannot be lost between the two documents.</t>
         </is>
       </c>
     </row>
@@ -3203,7 +3203,7 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>The 'Monthly demand by project' pop-up now states THE MONTH'S TOTAL across every project in view, under a rule, and the band's share of it - the two things 'Monthly demand by person' already carried and this one did not. A band read on its own cannot say whether the month came to five FTE or to fifty. Sheet 10 Graph 1 updated. No change to any figure: the total is the sum the chart was already drawing, and it is the same figure Graph 2 states for that month summed along the other axis - test_charts.py now holds the two to agreeing in WORDS as well as in pixels, month for month.</t>
+          <t>The 'Monthly demand by project' pop-up now states THE MONTH'S TOTAL across every project in view, under a rule, and the band's share of it - the two things 'Monthly demand by person' already carried and this one did not. A band read on its own cannot say whether the month came to five FTE or to fifty. Sheet 10 Graph 1 updated. No change to any figure: the total is the sum the chart was already drawing, and it is the same figure Graph 2 states for that month summed along the other axis - test_charts.py now holds the two to agreeing in WORDS as well as in pixels, month for month. Written against plan v2.42.</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
@@ -3976,7 +3976,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>PRAP_Development_Plan_v2.41.xlsx</t>
+          <t>PRAP_Development_Plan_v2.42.xlsx</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">

</xml_diff>